<commit_message>
Auto-actualizacion SAT Rio V [2026-09-28 12:15 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.63</v>
@@ -811,7 +811,7 @@
         <v>3.8</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>7.8</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-28 12:38 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -691,11 +691,11 @@
         <v>1.7</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
         <v>3.8</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -871,11 +871,11 @@
         <v>7.8</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-28 13:03 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.63</v>
@@ -695,7 +695,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -811,11 +811,11 @@
         <v>3.8</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -871,7 +871,7 @@
         <v>7.8</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0.3</v>

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-28 19:50 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -691,11 +691,11 @@
         <v>1.7</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>13.9</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0.96</v>
@@ -734,7 +734,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -811,11 +811,11 @@
         <v>3.8</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>13.9</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1.76</v>
+        <v>1.77</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>1.75</v>
@@ -871,11 +871,11 @@
         <v>7.8</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1.15</v>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0.67</v>
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0.3</v>

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-28 23:59 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1.34</v>
@@ -691,11 +691,11 @@
         <v>1.7</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>13.9</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.99</v>
+        <v>1.04</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0.96</v>
@@ -811,11 +811,11 @@
         <v>3.8</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>13.9</t>
+          <t>13.6</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1.15</v>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0.67</v>
@@ -974,7 +974,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-29 00:29 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -433,23 +433,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="27" customWidth="1" min="14" max="14"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="27" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,60 +467,70 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Tramo Jurisdiccional</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Nivel Actual (m)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Media Histórica (m)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Cota Alerta (m)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Cota Evacuación (m)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Margen Alerta (m)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Estado Semáforo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Tendencia Río</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Estación Meteo Cercana</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Distancia (km)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Lluvia 24h (mm)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Temp (°C)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Tiempo Viaje a LP (días)</t>
         </is>
@@ -535,50 +547,58 @@
           <t>Afluente Río Quinto</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>0.63</v>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Media (Córdoba)</t>
+        </is>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.63</v>
       </c>
       <c r="E2" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>1.9</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>2.4</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Vicuña Mackenna (Córdoba)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="M2" s="2" t="n">
         <v>5.8</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>S/D</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -595,50 +615,58 @@
           <t>Cuenca Río Quinto</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Media (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>1.33</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="E3" s="2" t="n">
         <v>1.34</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>2.4</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Hipólito Bouchard (Córdoba)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="M3" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>S/D</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -655,50 +683,58 @@
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>0.13</v>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Alta (San Luis)</t>
+        </is>
       </c>
       <c r="D4" s="2" t="n">
         <v>0.11</v>
       </c>
       <c r="E4" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F4" s="2" t="n">
         <v>2.5</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>3.2</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
+      <c r="H4" s="2" t="n">
+        <v>2.39</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Bajando ▼</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>Villa Reynolds (San Luis)</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="M4" s="2" t="n">
         <v>1.7</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>0.1</v>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>13.5</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -715,50 +751,58 @@
           <t>Río Quinto / Canal Devoto</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Media (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>1.04</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="E5" s="2" t="n">
         <v>0.96</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>2.8</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>3.4</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Creciendo ▲</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Río Bamba (Córdoba)</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="M5" s="2" t="n">
         <v>29.4</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="N5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>S/D</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -775,50 +819,58 @@
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>1.09</v>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Alta (San Luis)</t>
+        </is>
       </c>
       <c r="D6" s="2" t="n">
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="F6" s="2" t="n">
         <v>2.8</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>3.5</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Villa Mercedes (San Luis)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="M6" s="2" t="n">
         <v>3.8</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>0.1</v>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>13.6</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -835,50 +887,58 @@
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Alta (San Luis)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>1.77</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="E7" s="2" t="n">
         <v>1.75</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>2.9</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>3.6</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Justo Daract (San Luis)</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="M7" s="2" t="n">
         <v>7.8</v>
       </c>
-      <c r="L7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>14.3</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -895,50 +955,58 @@
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Media (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>1.14</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="E8" s="2" t="n">
         <v>1.15</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>2.6</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>3.2</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Nicolás Bruzzone (Córdoba)</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="M8" s="2" t="n">
         <v>25.1</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>S/D</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -955,50 +1023,58 @@
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Ingreso Cuenca Baja (La Pampa)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
         <v>0.68</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="E9" s="2" t="n">
         <v>0.67</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>2.2</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>2.8</v>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Creciendo ▲</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Hipólito Bouchard (Córdoba)</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="M9" s="2" t="n">
         <v>14.4</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>S/D</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -1015,50 +1091,58 @@
           <t>Río Trapiche (Afluente)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>0.3</v>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Cuenca Alta (San Luis)</t>
+        </is>
       </c>
       <c r="D10" s="2" t="n">
         <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F10" s="2" t="n">
         <v>1.8</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>2.3</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia Ordinaria</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>El Trapiche (San Luis)</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="M10" s="2" t="n">
         <v>0.6</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>11.6</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-29 04:47 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.33</v>
+        <v>1.34</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.34</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.11</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.39</v>
+        <v>2.45</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.04</v>
+        <v>0.96</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.76</v>
+        <v>1.84</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -863,11 +863,11 @@
         <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>13.6</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.1</v>
+        <v>1.5</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>14.8</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -964,7 +964,7 @@
         <v>1.14</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2.6</v>
@@ -1029,10 +1029,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.2</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.52</v>
+        <v>1.54</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1135,11 +1135,11 @@
         <v>0.6</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-29 10:56 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.34</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.11</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.45</v>
+        <v>2.49</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.97</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.84</v>
+        <v>1.83</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -863,11 +863,11 @@
         <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,10 +893,10 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.77</v>
+        <v>1.79</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1.75</v>
+        <v>1.76</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2.9</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.13</v>
+        <v>1.11</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>14.8</t>
+          <t>10.7</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.54</v>
+        <v>1.55</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1135,11 +1135,11 @@
         <v>0.6</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-29 16:44 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.63</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -689,10 +689,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2.5</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.49</v>
+        <v>2.51</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>18.3</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.97</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.83</v>
+        <v>1.86</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -846,7 +846,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>17.7</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>10.7</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.65</v>
+        <v>0.63</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.55</v>
+        <v>1.57</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-29 21:05 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.63</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.26</v>
+        <v>1.25</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-0.01</v>
+        <v>0.1</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.51</v>
+        <v>2.4</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>18.3</t>
+          <t>17.6</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.97</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.86</v>
+        <v>1.85</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -846,7 +846,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>17.7</t>
+          <t>18.1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.79</v>
+        <v>1.77</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.76</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>19.6</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>15.6</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-30 00:22 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.63</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.4</v>
+        <v>2.41</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>17.6</t>
+          <t>10.9</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
         <v>0.95</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.05</v>
+        <v>1.07</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.76</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>19.6</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-30 05:48 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>10.9</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.96</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.76</v>
+        <v>1.74</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.76</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.14</v>
+        <v>1.16</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>14.5</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.63</v>
+        <v>0.67</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.57</v>
+        <v>1.53</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-30 11:25 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.34</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>12.6</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.84</v>
+        <v>1.81</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.76</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.16</v>
+        <v>1.15</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>12.7</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.47</v>
+        <v>1.46</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-30 16:55 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.63</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>12.6</t>
+          <t>22.5</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.99</v>
+        <v>1.03</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.97</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.81</v>
+        <v>1.77</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.75</v>
+        <v>1.77</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.76</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.15</v>
+        <v>1.13</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>12.7</t>
+          <t>21.3</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.14</v>
+        <v>1.15</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.54</v>
+        <v>1.55</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.48</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-09-30 21:08 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.34</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.41</v>
+        <v>2.4</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>22.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.03</v>
+        <v>0.99</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.97</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.77</v>
+        <v>1.81</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.07</v>
@@ -837,7 +837,7 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.72</v>
+        <v>1.73</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -863,11 +863,11 @@
         <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>21.3</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>13.9</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 00:32 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.63</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.34</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -863,11 +863,11 @@
         <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.45</v>
+        <v>1.43</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.3</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1135,11 +1135,11 @@
         <v>0.6</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>13.9</t>
+          <t>7.7</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 06:29 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1.9</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.24</v>
+        <v>1.23</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.35</v>
+        <v>1.38</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.34</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.99</v>
+        <v>1.05</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.81</v>
+        <v>1.75</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.07</v>
@@ -837,7 +837,7 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.76</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.17</v>
+        <v>1.18</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.43</v>
+        <v>1.42</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>0.65</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>0.66</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.2</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,10 +1097,10 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1.8</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1135,11 +1135,11 @@
         <v>0.6</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.6</v>
+        <v>0.1</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>7.7</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 12:12 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -444,7 +444,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.64</v>
@@ -565,11 +565,11 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.38</v>
+        <v>1.4</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2.4</v>
@@ -633,16 +633,16 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,11 +701,11 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.39</v>
+        <v>2.38</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -715,23 +715,23 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Villa Reynolds (San Luis)</t>
+          <t>Presa El Chañar (Córdoba)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>REM San Luis</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1.7</v>
+        <v>38.6</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>S/D</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.98</v>
@@ -769,16 +769,16 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.75</v>
+        <v>1.79</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.07</v>
@@ -837,11 +837,11 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.72</v>
+        <v>1.73</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -851,23 +851,23 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Villa Mercedes (San Luis)</t>
+          <t>Chaján (Córdoba)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>REM San Luis</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>3.8</v>
+        <v>50.2</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>S/D</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -919,23 +919,23 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Justo Daract (San Luis)</t>
+          <t>Presa El Chañar (Córdoba)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>REM San Luis</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>7.8</v>
+        <v>10.1</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>S/D</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,11 +1041,11 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.56</v>
+        <v>1.57</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.31</v>
@@ -1109,11 +1109,11 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Ordinaria</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1123,23 +1123,23 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>El Trapiche (San Luis)</t>
+          <t>Chaján (Córdoba)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>REM San Luis</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.6</v>
+        <v>110</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>7.8</t>
+          <t>S/D</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 13:47 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.64</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.38</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.35</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -715,23 +715,23 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Presa El Chañar (Córdoba)</t>
+          <t>Villa Reynolds (San Luis)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>REM San Luis</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>38.6</v>
+        <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>S/D</t>
+          <t>15.8</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -851,23 +851,23 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Chaján (Córdoba)</t>
+          <t>Villa Mercedes (San Luis)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>REM San Luis</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>50.2</v>
+        <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>S/D</t>
+          <t>15.1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
         <v>1.78</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1.76</v>
+        <v>1.77</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2.9</v>
@@ -919,23 +919,23 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Presa El Chañar (Córdoba)</t>
+          <t>Justo Daract (San Luis)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>REM San Luis</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>10.1</v>
+        <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>S/D</t>
+          <t>15.2</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1123,23 +1123,23 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Chaján (Córdoba)</t>
+          <t>El Trapiche (San Luis)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>REM San Luis</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>110</v>
+        <v>0.6</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>S/D</t>
+          <t>12.4</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 15:22 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -457,12 +457,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Estación Hidrológica</t>
+          <t>Estacion Hidrologica</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Río / Cuenca</t>
+          <t>Rio / Cuenca</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -477,7 +477,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Media Histórica (m)</t>
+          <t>Media Historica (m)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Cota Evacuación (m)</t>
+          <t>Cota Evacuacion (m)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -497,17 +497,17 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Estado Semáforo</t>
+          <t>Estado Semaforo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Tendencia Río</t>
+          <t>Tendencia Rio</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Estación Meteo Cercana</t>
+          <t>Estacion Meteo Cercana</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -527,29 +527,29 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Temp (°C)</t>
+          <t>Temp (C)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Tiempo Viaje a LP (días)</t>
+          <t>Tiempo Viaje a LP (dias)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aº El Aji - RN Nº35 y RN Nº7</t>
+          <t>Ao El Aji - RN No35 y RN No7</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Afluente Río Quinto</t>
+          <t>Afluente Rio Quinto</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Córdoba)</t>
+          <t>Cuenca Media (Cordoba)</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -569,22 +569,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Vicuña Mackenna (Córdoba)</t>
+          <t>Vicuna Mackenna (Cordoba)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>Omixom Cordoba</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
@@ -612,12 +612,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Río Quinto</t>
+          <t>Cuenca Rio Quinto</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Córdoba)</t>
+          <t>Cuenca Media (Cordoba)</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -637,22 +637,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Bajando -</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Hipólito Bouchard (Córdoba)</t>
+          <t>Hipolito Bouchard (Cordoba)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>Omixom Cordoba</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -675,12 +675,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Quinto - Av Circunvalación</t>
+          <t>Quinto - Av Circunvalacion</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Río Quinto</t>
+          <t>Rio Quinto</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -695,22 +695,22 @@
         <v>0.1</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>3.2</v>
+        <v>2.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.38</v>
+        <v>1.48</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>15.8</t>
+          <t>18.1</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -748,16 +748,16 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Río Quinto / Canal Devoto</t>
+          <t>Rio Quinto / Canal Devoto</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Córdoba)</t>
+          <t>Cuenca Media (Cordoba)</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.98</v>
@@ -769,26 +769,26 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Río Bamba (Córdoba)</t>
+          <t>Rio Bamba (Cordoba)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>Omixom Cordoba</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
@@ -816,7 +816,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Río Quinto</t>
+          <t>Rio Quinto</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.07</v>
@@ -837,16 +837,16 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>15.1</t>
+          <t>16.2</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Río Quinto</t>
+          <t>Rio Quinto</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -909,12 +909,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>15.2</t>
+          <t>16.8</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -952,16 +952,16 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Río Quinto</t>
+          <t>Rio Quinto</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Córdoba)</t>
+          <t>Cuenca Media (Cordoba)</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.18</v>
+        <v>1.19</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,26 +973,26 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.42</v>
+        <v>1.41</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Nicolás Bruzzone (Córdoba)</t>
+          <t>Nicolas Bruzzone (Cordoba)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>Omixom Cordoba</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
@@ -1015,12 +1015,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Quinto - RP Nº26</t>
+          <t>Quinto - RP No26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Río Quinto</t>
+          <t>Rio Quinto</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,22 +1045,22 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Hipólito Bouchard (Córdoba)</t>
+          <t>Hipolito Bouchard (Cordoba)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Omixom Córdoba</t>
+          <t>Omixom Cordoba</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Río Trapiche (Afluente)</t>
+          <t>Rio Trapiche (Afluente)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1113,12 +1113,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
+          <t>Vigilancia Preventiva / Calma Hidrologica</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>12.4</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 18:50 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Bajando -</t>
+          <t>Estable =</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>18.8</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>16.2</t>
+          <t>18.3</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.77</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>16.8</t>
+          <t>17.1</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.19</v>
+        <v>1.18</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.14</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.31</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 19:05 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>18.8</t>
+          <t>18.9</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.07</v>
@@ -837,7 +837,7 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.72</v>
+        <v>1.73</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>18.3</t>
+          <t>19.1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>17.5</t>
+          <t>17.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 19:31 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -457,12 +457,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Estacion Hidrologica</t>
+          <t>Estación Hidrológica</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Rio / Cuenca</t>
+          <t>Río / Cuenca</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -477,7 +477,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Media Historica (m)</t>
+          <t>Media Histórica (m)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Cota Evacuacion (m)</t>
+          <t>Cota Evacuación (m)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -497,17 +497,17 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Estado Semaforo</t>
+          <t>Estado Semáforo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Tendencia Rio</t>
+          <t>Tendencia Río</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Estacion Meteo Cercana</t>
+          <t>Estación Meteo Cercana</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -527,29 +527,29 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Temp (C)</t>
+          <t>Temp (°C)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Tiempo Viaje a LP (dias)</t>
+          <t>Tiempo Viaje a LP (días)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ao El Aji - RN No35 y RN No7</t>
+          <t>Aº El Aji - RN Nº35 y RN Nº7</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Afluente Rio Quinto</t>
+          <t>Afluente Río Quinto</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Cordoba)</t>
+          <t>Cuenca Media (Córdoba)</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -569,22 +569,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Vicuna Mackenna (Cordoba)</t>
+          <t>Vicuña Mackenna (Córdoba)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Omixom Cordoba</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
@@ -612,12 +612,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Rio Quinto</t>
+          <t>Cuenca Río Quinto</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Cordoba)</t>
+          <t>Cuenca Media (Córdoba)</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -637,22 +637,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Hipolito Bouchard (Cordoba)</t>
+          <t>Hipólito Bouchard (Córdoba)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Omixom Cordoba</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -675,12 +675,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Quinto - Av Circunvalacion</t>
+          <t>Quinto - Av Circunvalación</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Rio Quinto</t>
+          <t>Río Quinto</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -695,22 +695,22 @@
         <v>0.1</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1.48</v>
+        <v>2.38</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>18.9</t>
+          <t>18.7</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Rio Quinto / Canal Devoto</t>
+          <t>Río Quinto / Canal Devoto</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Cordoba)</t>
+          <t>Cuenca Media (Córdoba)</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -773,22 +773,22 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Rio Bamba (Cordoba)</t>
+          <t>Río Bamba (Córdoba)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Omixom Cordoba</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
@@ -816,7 +816,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Rio Quinto</t>
+          <t>Río Quinto</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -841,12 +841,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>19.1</t>
+          <t>18.9</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Rio Quinto</t>
+          <t>Río Quinto</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -909,12 +909,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Rio Quinto</t>
+          <t>Río Quinto</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Media (Cordoba)</t>
+          <t>Cuenca Media (Córdoba)</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -977,22 +977,22 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Nicolas Bruzzone (Cordoba)</t>
+          <t>Nicolás Bruzzone (Córdoba)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Omixom Cordoba</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
@@ -1015,12 +1015,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Quinto - RP No26</t>
+          <t>Quinto - RP Nº26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Rio Quinto</t>
+          <t>Río Quinto</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,22 +1045,22 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Hipolito Bouchard (Cordoba)</t>
+          <t>Hipólito Bouchard (Córdoba)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Omixom Cordoba</t>
+          <t>Omixom Córdoba</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Rio Trapiche (Afluente)</t>
+          <t>Río Trapiche (Afluente)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1113,12 +1113,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Vigilancia Preventiva / Calma Hidrologica</t>
+          <t>Vigilancia Preventiva / Calma Hidrológica</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Estable =</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>17.8</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-01 23:08 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.38</v>
+        <v>1.37</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.35</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>18.7</t>
+          <t>11.8</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.98</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.8</v>
+        <v>1.79</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>18.9</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -961,10 +961,10 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1.14</v>
+        <v>1.15</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2.6</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.42</v>
+        <v>1.44</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.57</v>
+        <v>1.56</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.31</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-02 02:11 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.64</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.07</v>
@@ -837,7 +837,7 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.15</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.44</v>
+        <v>1.43</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.64</v>
+        <v>0.66</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.56</v>
+        <v>1.54</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-02 08:36 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -556,7 +556,7 @@
         <v>0.68</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1.9</v>
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2.4</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.01</v>
+        <v>1.04</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.79</v>
+        <v>1.76</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>12.5</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.77</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.15</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.54</v>
+        <v>1.53</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1097,10 +1097,10 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1.8</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-02 14:58 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.65</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>20.1</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.99</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.76</v>
+        <v>1.78</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>20.7</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.53</v>
+        <v>1.51</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>18.2</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-02 19:46 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.38</v>
+        <v>1.44</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.36</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.38</v>
+        <v>2.37</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>20.1</t>
+          <t>22.9</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.99</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.8</v>
+        <v>1.79</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.77</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>17.1</t>
+          <t>22.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.51</v>
+        <v>1.48</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>18.2</t>
+          <t>19.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-02 23:18 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.44</v>
+        <v>1.4</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.36</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>22.9</t>
+          <t>20.9</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0.99</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>21.3</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
         <v>1.79</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2.9</v>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>22.5</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.65</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>19.8</t>
+          <t>12.6</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-03 02:05 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.65</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.38</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.36</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>20.9</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>21.3</t>
+          <t>20.6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.79</v>
+        <v>1.78</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.78</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.15</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.44</v>
+        <v>1.43</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1032,7 +1032,7 @@
         <v>0.71</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.2</v>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>12.6</t>
+          <t>16.7</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-03 08:01 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -556,7 +556,7 @@
         <v>0.68</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1.9</v>
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.38</v>
+        <v>1.36</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2.4</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.02</v>
+        <v>1.04</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -863,11 +863,11 @@
         <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>20.6</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.78</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>12.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -964,7 +964,7 @@
         <v>1.17</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1.15</v>
+        <v>1.16</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2.6</v>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>16.7</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-03 13:14 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.37</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>17.3</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1</v>
+        <v>1.04</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.8</v>
+        <v>1.76</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1.06</v>
@@ -837,7 +837,7 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -863,11 +863,11 @@
         <v>3.8</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>16.6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -931,11 +931,11 @@
         <v>7.8</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>16.9</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.17</v>
+        <v>1.18</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.16</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.43</v>
+        <v>1.42</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-03 17:21 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.37</v>
+        <v>1.36</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.37</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.1</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -727,11 +727,11 @@
         <v>1.7</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>17.3</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.76</v>
+        <v>1.78</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>16.6</t>
+          <t>21.2</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>16.9</t>
+          <t>21.3</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.5</v>
+        <v>1.51</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>17.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-03 20:00 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.78</v>
+        <v>1.8</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -837,7 +837,7 @@
         <v>3.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>21.2</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>21.3</t>
+          <t>21.9</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>17.8</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-03 22:47 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.66</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.37</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>15.6</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.8</v>
+        <v>1.79</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>17.9</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>21.9</t>
+          <t>16.1</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.51</v>
+        <v>1.53</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>12.7</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-04 02:01 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -692,7 +692,7 @@
         <v>0.14</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2.5</v>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.79</v>
+        <v>1.77</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>17.9</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>16.1</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.66</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>12.7</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-04 08:22 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -556,7 +556,7 @@
         <v>0.67</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1.9</v>
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2.4</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         <v>0.14</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2.5</v>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.77</v>
+        <v>1.79</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
         <v>1.08</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.8</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.79</v>
+        <v>1.78</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.78</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -964,7 +964,7 @@
         <v>1.18</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2.6</v>
@@ -1029,10 +1029,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.2</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.52</v>
+        <v>1.51</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-04 14:14 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.67</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.12</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>22.3</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.01</v>
+        <v>1.06</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1.01</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.79</v>
+        <v>1.74</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>19.6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.78</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>22.7</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.49</v>
+        <v>1.51</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-04 18:12 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>22.3</t>
+          <t>23.5</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.06</v>
+        <v>1.02</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1.01</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.74</v>
+        <v>1.78</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>19.6</t>
+          <t>23.6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>22.7</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.17</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>20.7</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-04 21:32 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.67</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.38</v>
+        <v>1.4</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.38</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.12</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>23.5</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1.01</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.78</v>
+        <v>1.81</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>23.6</t>
+          <t>18.2</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.79</v>
+        <v>1.78</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1.78</v>
@@ -905,7 +905,7 @@
         <v>3.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.17</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.71</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.67</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Creciendo ▲</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>17.9</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-05 00:09 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.67</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.12</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>18.2</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.17</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.44</v>
+        <v>1.43</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Creciendo ▲</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0.32</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.5</v>
+        <v>1.51</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>17.9</t>
+          <t>16.8</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-05 05:31 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1.38</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>1.04</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,10 +689,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>0.13</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0.12</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2.5</v>
@@ -701,7 +701,7 @@
         <v>3.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>14.5</t>
+          <t>15.8</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.8</v>
@@ -769,7 +769,7 @@
         <v>3.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.81</v>
+        <v>1.8</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Estable ▬</t>
+          <t>Bajando ▼</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>15.6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
         <v>1.78</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2.9</v>
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>12.6</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1029,10 +1029,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.2</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1097,10 +1097,10 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1.8</v>
@@ -1109,7 +1109,7 @@
         <v>2.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>16.8</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualizacion SAT Rio V [2026-10-05 12:36 UTC]
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.67</v>
@@ -565,7 +565,7 @@
         <v>2.4</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>15.8</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Bajando ▼</t>
+          <t>Estable ▬</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>14.9</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>12.6</t>
+          <t>15.7</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1.17</v>
@@ -973,7 +973,7 @@
         <v>3.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.68</v>
@@ -1041,7 +1041,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>12.4</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 10:55 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cruce Hidro-Meteo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cruce Hidrometeorológico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,29 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -62,12 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,716 +413,598 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="27" customWidth="1" min="16" max="16"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Estación Hidrológica</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Río / Cuenca</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Tramo Jurisdiccional</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Nivel Actual (m)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Media Histórica (m)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Cota Alerta (m)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Cota Evacuación (m)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Margen Alerta (m)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Estado Semáforo</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tendencia Río</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Estación Meteo Cercana</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Distancia (km)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Lluvia 24h (mm)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Temp (°C)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Tiempo Viaje a LP (días)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Aº El Aji - RN Nº35 y RN Nº7</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Afluente Río Quinto</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Media (Córdoba)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" t="n">
         <v>0.65</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="D2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="E2" t="n">
         <v>1.9</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="F2" t="n">
         <v>2.4</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="G2" t="n">
         <v>1.25</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Vicuña Mackenna (Córdoba)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="L2" t="n">
         <v>5.8</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Laguna La Margarita</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Cuenca Río Quinto</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Media (Córdoba)</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" t="n">
         <v>1.36</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="D3" t="n">
         <v>1.38</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="E3" t="n">
         <v>2.4</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="F3" t="n">
         <v>3</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="G3" t="n">
         <v>1.04</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Hipólito Bouchard (Córdoba)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="L3" t="n">
         <v>21</v>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="M3" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Quinto - Av Circunvalación</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Alta (San Luis)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="C4" t="n">
         <v>0.13</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="D4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E4" t="n">
         <v>2.5</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="F4" t="n">
         <v>3.2</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="G4" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Villa Reynolds (San Luis)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="L4" t="n">
         <v>1.7</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="M4" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>14.3</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Quinto - Canal Devoto RP 4</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Río Quinto / Canal Devoto</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Media (Córdoba)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="F5" s="2" t="n">
+      <c r="C5" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="E5" t="n">
         <v>2.8</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="F5" t="n">
         <v>3.4</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="G5" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Bajando ▼</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Río Bamba (Córdoba)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="L5" t="n">
         <v>29.4</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="M5" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Quinto - Dique Villa Mercedes</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Alta (San Luis)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="F6" s="2" t="n">
+      <c r="C6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E6" t="n">
         <v>2.8</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="F6" t="n">
         <v>3.5</v>
       </c>
-      <c r="H6" s="2" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="G6" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Villa Mercedes (San Luis)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="L6" t="n">
         <v>3.8</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="M6" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>14.9</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Quinto - Justo Daract</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Alta (San Luis)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="C7" t="n">
         <v>1.78</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="D7" t="n">
         <v>1.79</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="E7" t="n">
         <v>2.9</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="F7" t="n">
         <v>3.6</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="G7" t="n">
         <v>1.12</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Justo Daract (San Luis)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="L7" t="n">
         <v>7.8</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="M7" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>15.7</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Quinto - R.N. 35</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Media (Córdoba)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="E8" s="2" t="n">
+      <c r="C8" t="n">
         <v>1.17</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="D8" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="E8" t="n">
         <v>2.6</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="F8" t="n">
         <v>3.2</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="G8" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Nicolás Bruzzone (Córdoba)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="L8" t="n">
         <v>25.1</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="M8" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Quinto - RP Nº26</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Río Quinto</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Ingreso Cuenca Baja (La Pampa)</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="F9" s="2" t="n">
+      <c r="C9" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E9" t="n">
         <v>2.2</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="F9" t="n">
         <v>2.8</v>
       </c>
-      <c r="H9" s="2" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="G9" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Hipólito Bouchard (Córdoba)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Omixom Córdoba</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="L9" t="n">
         <v>14.4</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="M9" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Trapiche - Hosteria El Trapiche</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Río Trapiche (Afluente)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Cuenca Alta (San Luis)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="C10" t="n">
         <v>0.3</v>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="F10" s="2" t="n">
+      <c r="D10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E10" t="n">
         <v>1.8</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="F10" t="n">
         <v>2.3</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="G10" t="n">
         <v>1.5</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Vigilancia Preventiva / Calma Hidrológica</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Normal / Seguro</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Estable ▬</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>El Trapiche (San Luis)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>REM San Luis</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="L10" t="n">
         <v>0.6</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="M10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>12.4</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 12:37 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cruce Hidrometeorológico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cruce Cuenca Rio V" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Río / Cuenca</t>
+          <t>Río</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -434,57 +434,32 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Media Histórica (m)</t>
+          <t>Cota Alerta (m)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Cota Alerta (m)</t>
+          <t>Cota Evac (m)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Cota Evacuación (m)</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Margen Alerta (m)</t>
+          <t>Meteo Cercana</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Estado Semáforo</t>
+          <t>Lluvia 24h (mm)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Tendencia Río</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Estación Meteo Cercana</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Distancia (km)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Lluvia 24h (mm)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Tiempo Viaje a LP (días)</t>
+          <t>Ventana Onda LP</t>
         </is>
       </c>
     </row>
@@ -500,47 +475,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="D2" t="n">
-        <v>0.66</v>
+        <v>1.9</v>
       </c>
       <c r="E2" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="F2" t="n">
         <v>2.4</v>
       </c>
-      <c r="G2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Vicuña Mackenna</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Vicuña Mackenna (Córdoba)</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Omixom Córdoba</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -561,44 +517,25 @@
         <v>1.36</v>
       </c>
       <c r="D3" t="n">
-        <v>1.38</v>
+        <v>2.4</v>
       </c>
       <c r="E3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="F3" t="n">
         <v>3</v>
       </c>
-      <c r="G3" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Hipólito Bouchard</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Hipólito Bouchard (Córdoba)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Omixom Córdoba</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>21</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -619,44 +556,25 @@
         <v>0.13</v>
       </c>
       <c r="D4" t="n">
-        <v>0.13</v>
+        <v>2.5</v>
       </c>
       <c r="E4" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F4" t="n">
         <v>3.2</v>
       </c>
-      <c r="G4" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Villa Reynolds</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Villa Reynolds (San Luis)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>REM San Luis</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -677,44 +595,25 @@
         <v>0.99</v>
       </c>
       <c r="D5" t="n">
-        <v>1.01</v>
+        <v>2.8</v>
       </c>
       <c r="E5" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="F5" t="n">
         <v>3.4</v>
       </c>
-      <c r="G5" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Río Bamba</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="inlineStr">
-        <is>
-          <t>Bajando ▼</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Río Bamba (Córdoba)</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Omixom Córdoba</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -735,44 +634,25 @@
         <v>1.1</v>
       </c>
       <c r="D6" t="n">
-        <v>1.07</v>
+        <v>2.8</v>
       </c>
       <c r="E6" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="F6" t="n">
         <v>3.5</v>
       </c>
-      <c r="G6" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Villa Mercedes</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Villa Mercedes (San Luis)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>REM San Luis</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -793,44 +673,25 @@
         <v>1.78</v>
       </c>
       <c r="D7" t="n">
-        <v>1.79</v>
+        <v>2.9</v>
       </c>
       <c r="E7" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="F7" t="n">
         <v>3.6</v>
       </c>
-      <c r="G7" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Justo Daract</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Justo Daract (San Luis)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>REM San Luis</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -848,47 +709,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="D8" t="n">
-        <v>1.17</v>
+        <v>2.6</v>
       </c>
       <c r="E8" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F8" t="n">
         <v>3.2</v>
       </c>
-      <c r="G8" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Nicolás Bruzzone</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Nicolás Bruzzone (Córdoba)</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Omixom Córdoba</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>25.1</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -909,44 +751,25 @@
         <v>0.67</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.2</v>
       </c>
       <c r="E9" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="F9" t="n">
         <v>2.8</v>
       </c>
-      <c r="G9" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Hipólito Bouchard</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Hipólito Bouchard (Córdoba)</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Omixom Córdoba</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>
@@ -967,44 +790,25 @@
         <v>0.3</v>
       </c>
       <c r="D10" t="n">
-        <v>0.3</v>
+        <v>1.8</v>
       </c>
       <c r="E10" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F10" t="n">
         <v>2.3</v>
       </c>
-      <c r="G10" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Normal / Seguro</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>El Trapiche</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" t="inlineStr">
-        <is>
-          <t>Estable ▬</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>El Trapiche (San Luis)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>REM San Luis</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="inlineStr">
         <is>
           <t>7-10 d</t>
         </is>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 13:06 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Cruce Cuenca Rio V" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pronostico ECMWF 72h" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="D2" t="n">
         <v>1.9</v>
@@ -514,7 +515,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="D3" t="n">
         <v>2.4</v>
@@ -787,7 +788,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D10" t="n">
         <v>1.8</v>
@@ -812,6 +813,300 @@
         <is>
           <t>7-10 d</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Nodo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Provincia</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Lluvia Hoy (mm)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>+24h (mm)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>+48h (mm)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Acumulado 72h (mm)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Media Mensual (mm)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Media Anual (mm)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>% Aporte Mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Villa Mercedes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>San Luis</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cabecera / Nacientes</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>55</v>
+      </c>
+      <c r="I2" t="n">
+        <v>680</v>
+      </c>
+      <c r="J2" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>General Levalle</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cuenca Media (Aporte)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I3" t="n">
+        <v>750</v>
+      </c>
+      <c r="J3" t="n">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jovita</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cuenca Media-Baja</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>70</v>
+      </c>
+      <c r="I4" t="n">
+        <v>770</v>
+      </c>
+      <c r="J4" t="n">
+        <v>23.9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Realicó</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>La Pampa</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Norte Pampeano (RN 35)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="H5" t="n">
+        <v>75</v>
+      </c>
+      <c r="I5" t="n">
+        <v>800</v>
+      </c>
+      <c r="J5" t="n">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Intendente Alvear</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>La Pampa</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Norte Pampeano (Meridiano V)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>78</v>
+      </c>
+      <c r="I6" t="n">
+        <v>820</v>
+      </c>
+      <c r="J6" t="n">
+        <v>19.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Punta Alta (Rancul)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>La Pampa</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Norte Pampeano (RP 9)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>72</v>
+      </c>
+      <c r="I7" t="n">
+        <v>780</v>
+      </c>
+      <c r="J7" t="n">
+        <v>13.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 13:50 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -898,16 +898,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5.1</v>
+        <v>2.8</v>
       </c>
       <c r="E2" t="n">
-        <v>8.9</v>
+        <v>11.7</v>
       </c>
       <c r="F2" t="n">
-        <v>3.6</v>
+        <v>2.7</v>
       </c>
       <c r="G2" t="n">
-        <v>17.6</v>
+        <v>17.2</v>
       </c>
       <c r="H2" t="n">
         <v>55</v>
@@ -916,7 +916,7 @@
         <v>680</v>
       </c>
       <c r="J2" t="n">
-        <v>32</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="3">
@@ -936,16 +936,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>16.3</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3.8</v>
       </c>
       <c r="G3" t="n">
-        <v>12.6</v>
+        <v>20.1</v>
       </c>
       <c r="H3" t="n">
         <v>68</v>
@@ -954,7 +954,7 @@
         <v>750</v>
       </c>
       <c r="J3" t="n">
-        <v>18.5</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="4">
@@ -974,16 +974,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>14.7</v>
+        <v>15.5</v>
       </c>
       <c r="F4" t="n">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
       <c r="G4" t="n">
-        <v>16.7</v>
+        <v>18.1</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -992,7 +992,7 @@
         <v>770</v>
       </c>
       <c r="J4" t="n">
-        <v>23.9</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="5">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>14.8</v>
+        <v>9.9</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>6.6</v>
       </c>
       <c r="G5" t="n">
-        <v>16.7</v>
+        <v>16.5</v>
       </c>
       <c r="H5" t="n">
         <v>75</v>
@@ -1030,7 +1030,7 @@
         <v>800</v>
       </c>
       <c r="J5" t="n">
-        <v>22.3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="E6" t="n">
-        <v>13.4</v>
+        <v>12.6</v>
       </c>
       <c r="F6" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="G6" t="n">
-        <v>15.5</v>
+        <v>14.5</v>
       </c>
       <c r="H6" t="n">
         <v>78</v>
@@ -1068,7 +1068,7 @@
         <v>820</v>
       </c>
       <c r="J6" t="n">
-        <v>19.9</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="7">
@@ -1088,16 +1088,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E7" t="n">
-        <v>7.1</v>
+        <v>10.7</v>
       </c>
       <c r="F7" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="G7" t="n">
-        <v>9.6</v>
+        <v>12.6</v>
       </c>
       <c r="H7" t="n">
         <v>72</v>
@@ -1106,7 +1106,7 @@
         <v>780</v>
       </c>
       <c r="J7" t="n">
-        <v>13.3</v>
+        <v>17.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 15:03 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="D2" t="n">
         <v>1.9</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="D4" t="n">
         <v>2.5</v>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 19:10 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="D3" t="n">
         <v>2.4</v>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="D5" t="n">
         <v>2.8</v>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="D7" t="n">
         <v>2.9</v>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="D10" t="n">
         <v>1.8</v>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 20:12 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="D2" t="n">
         <v>1.9</v>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="D6" t="n">
         <v>2.8</v>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
       <c r="D7" t="n">
         <v>2.9</v>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.16</v>
+        <v>1.15</v>
       </c>
       <c r="D8" t="n">
         <v>2.6</v>
@@ -898,16 +898,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.8</v>
+        <v>4.1</v>
       </c>
       <c r="E2" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="F2" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="G2" t="n">
-        <v>17.2</v>
+        <v>18.2</v>
       </c>
       <c r="H2" t="n">
         <v>55</v>
@@ -916,7 +916,7 @@
         <v>680</v>
       </c>
       <c r="J2" t="n">
-        <v>31.3</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="3">
@@ -939,13 +939,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>16.3</v>
+        <v>15.1</v>
       </c>
       <c r="F3" t="n">
-        <v>3.8</v>
+        <v>1.8</v>
       </c>
       <c r="G3" t="n">
-        <v>20.1</v>
+        <v>16.9</v>
       </c>
       <c r="H3" t="n">
         <v>68</v>
@@ -954,7 +954,7 @@
         <v>750</v>
       </c>
       <c r="J3" t="n">
-        <v>29.6</v>
+        <v>24.9</v>
       </c>
     </row>
     <row r="4">
@@ -977,13 +977,13 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>15.5</v>
+        <v>7.7</v>
       </c>
       <c r="F4" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="G4" t="n">
-        <v>18.1</v>
+        <v>10.8</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -992,7 +992,7 @@
         <v>770</v>
       </c>
       <c r="J4" t="n">
-        <v>25.9</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="5">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E5" t="n">
-        <v>9.9</v>
+        <v>3.6</v>
       </c>
       <c r="F5" t="n">
-        <v>6.6</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>16.5</v>
+        <v>5.8</v>
       </c>
       <c r="H5" t="n">
         <v>75</v>
@@ -1030,7 +1030,7 @@
         <v>800</v>
       </c>
       <c r="J5" t="n">
-        <v>22</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="6">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E6" t="n">
-        <v>12.6</v>
+        <v>24.5</v>
       </c>
       <c r="F6" t="n">
-        <v>1.1</v>
+        <v>3.5</v>
       </c>
       <c r="G6" t="n">
-        <v>14.5</v>
+        <v>29.1</v>
       </c>
       <c r="H6" t="n">
         <v>78</v>
@@ -1068,7 +1068,7 @@
         <v>820</v>
       </c>
       <c r="J6" t="n">
-        <v>18.6</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="7">
@@ -1088,16 +1088,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="E7" t="n">
-        <v>10.7</v>
+        <v>14.3</v>
       </c>
       <c r="F7" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="G7" t="n">
-        <v>12.6</v>
+        <v>17.2</v>
       </c>
       <c r="H7" t="n">
         <v>72</v>
@@ -1106,7 +1106,7 @@
         <v>780</v>
       </c>
       <c r="J7" t="n">
-        <v>17.5</v>
+        <v>23.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-06 23:53 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="D5" t="n">
         <v>2.8</v>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="D6" t="n">
         <v>2.8</v>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="D7" t="n">
         <v>2.9</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D9" t="n">
         <v>2.2</v>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D10" t="n">
         <v>1.8</v>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-07 03:36 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="D2" t="n">
         <v>1.9</v>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.38</v>
+        <v>1.43</v>
       </c>
       <c r="D3" t="n">
         <v>2.4</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="D4" t="n">
         <v>2.5</v>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.98</v>
+        <v>1.69</v>
       </c>
       <c r="D5" t="n">
         <v>2.8</v>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.77</v>
+        <v>1.79</v>
       </c>
       <c r="D7" t="n">
         <v>2.9</v>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.15</v>
+        <v>1.22</v>
       </c>
       <c r="D8" t="n">
         <v>2.6</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.78</v>
       </c>
       <c r="D9" t="n">
         <v>2.2</v>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.29</v>
+        <v>0.32</v>
       </c>
       <c r="D10" t="n">
         <v>1.8</v>
@@ -898,16 +898,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4.1</v>
+        <v>7.8</v>
       </c>
       <c r="E2" t="n">
-        <v>11.6</v>
+        <v>4.6</v>
       </c>
       <c r="F2" t="n">
-        <v>2.5</v>
+        <v>10.8</v>
       </c>
       <c r="G2" t="n">
-        <v>18.2</v>
+        <v>23.2</v>
       </c>
       <c r="H2" t="n">
         <v>55</v>
@@ -916,7 +916,7 @@
         <v>680</v>
       </c>
       <c r="J2" t="n">
-        <v>33.1</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="3">
@@ -936,16 +936,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>6.3</v>
       </c>
       <c r="E3" t="n">
-        <v>15.1</v>
+        <v>1.4</v>
       </c>
       <c r="F3" t="n">
-        <v>1.8</v>
+        <v>12.4</v>
       </c>
       <c r="G3" t="n">
-        <v>16.9</v>
+        <v>20.1</v>
       </c>
       <c r="H3" t="n">
         <v>68</v>
@@ -954,7 +954,7 @@
         <v>750</v>
       </c>
       <c r="J3" t="n">
-        <v>24.9</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="4">
@@ -974,16 +974,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>7.9</v>
       </c>
       <c r="E4" t="n">
-        <v>7.7</v>
+        <v>3.2</v>
       </c>
       <c r="F4" t="n">
-        <v>3.1</v>
+        <v>10.2</v>
       </c>
       <c r="G4" t="n">
-        <v>10.8</v>
+        <v>21.3</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -992,7 +992,7 @@
         <v>770</v>
       </c>
       <c r="J4" t="n">
-        <v>15.4</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="5">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.2</v>
+        <v>6.3</v>
       </c>
       <c r="E5" t="n">
-        <v>3.6</v>
+        <v>1.4</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>6.6</v>
       </c>
       <c r="G5" t="n">
-        <v>5.8</v>
+        <v>14.3</v>
       </c>
       <c r="H5" t="n">
         <v>75</v>
@@ -1030,7 +1030,7 @@
         <v>800</v>
       </c>
       <c r="J5" t="n">
-        <v>7.7</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="6">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.1</v>
+        <v>28</v>
       </c>
       <c r="E6" t="n">
-        <v>24.5</v>
+        <v>5.9</v>
       </c>
       <c r="F6" t="n">
-        <v>3.5</v>
+        <v>7.1</v>
       </c>
       <c r="G6" t="n">
-        <v>29.1</v>
+        <v>41</v>
       </c>
       <c r="H6" t="n">
         <v>78</v>
@@ -1068,7 +1068,7 @@
         <v>820</v>
       </c>
       <c r="J6" t="n">
-        <v>37.3</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="7">
@@ -1088,16 +1088,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>14.3</v>
+        <v>1.8</v>
       </c>
       <c r="F7" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G7" t="n">
-        <v>17.2</v>
+        <v>14.8</v>
       </c>
       <c r="H7" t="n">
         <v>72</v>
@@ -1106,7 +1106,7 @@
         <v>780</v>
       </c>
       <c r="J7" t="n">
-        <v>23.9</v>
+        <v>20.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-07 10:34 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="D2" t="n">
         <v>1.9</v>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.43</v>
+        <v>1.39</v>
       </c>
       <c r="D3" t="n">
         <v>2.4</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="D4" t="n">
         <v>2.5</v>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.69</v>
+        <v>0.98</v>
       </c>
       <c r="D5" t="n">
         <v>2.8</v>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="D6" t="n">
         <v>2.8</v>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.79</v>
+        <v>1.77</v>
       </c>
       <c r="D7" t="n">
         <v>2.9</v>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.22</v>
+        <v>1.15</v>
       </c>
       <c r="D8" t="n">
         <v>2.6</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.78</v>
+        <v>0.71</v>
       </c>
       <c r="D9" t="n">
         <v>2.2</v>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="D10" t="n">
         <v>1.8</v>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -898,16 +898,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7.8</v>
+        <v>8.4</v>
       </c>
       <c r="E2" t="n">
-        <v>4.6</v>
+        <v>1.9</v>
       </c>
       <c r="F2" t="n">
-        <v>10.8</v>
+        <v>14.7</v>
       </c>
       <c r="G2" t="n">
-        <v>23.2</v>
+        <v>25</v>
       </c>
       <c r="H2" t="n">
         <v>55</v>
@@ -916,7 +916,7 @@
         <v>680</v>
       </c>
       <c r="J2" t="n">
-        <v>42.2</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="3">
@@ -936,16 +936,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6.3</v>
+        <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="F3" t="n">
-        <v>12.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>20.1</v>
+        <v>19.8</v>
       </c>
       <c r="H3" t="n">
         <v>68</v>
@@ -954,7 +954,7 @@
         <v>750</v>
       </c>
       <c r="J3" t="n">
-        <v>29.6</v>
+        <v>29.1</v>
       </c>
     </row>
     <row r="4">
@@ -974,16 +974,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>7.9</v>
+        <v>16.9</v>
       </c>
       <c r="E4" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="F4" t="n">
-        <v>10.2</v>
+        <v>3.6</v>
       </c>
       <c r="G4" t="n">
-        <v>21.3</v>
+        <v>22.8</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -992,7 +992,7 @@
         <v>770</v>
       </c>
       <c r="J4" t="n">
-        <v>30.4</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="5">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6.3</v>
+        <v>16.8</v>
       </c>
       <c r="E5" t="n">
-        <v>1.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>6.6</v>
+        <v>4.1</v>
       </c>
       <c r="G5" t="n">
-        <v>14.3</v>
+        <v>29.6</v>
       </c>
       <c r="H5" t="n">
         <v>75</v>
@@ -1030,7 +1030,7 @@
         <v>800</v>
       </c>
       <c r="J5" t="n">
-        <v>19.1</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="6">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>16.5</v>
       </c>
       <c r="E6" t="n">
-        <v>5.9</v>
+        <v>13.9</v>
       </c>
       <c r="F6" t="n">
-        <v>7.1</v>
+        <v>4.9</v>
       </c>
       <c r="G6" t="n">
-        <v>41</v>
+        <v>35.3</v>
       </c>
       <c r="H6" t="n">
         <v>78</v>
@@ -1068,7 +1068,7 @@
         <v>820</v>
       </c>
       <c r="J6" t="n">
-        <v>52.6</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="7">
@@ -1088,16 +1088,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8.699999999999999</v>
+        <v>17.3</v>
       </c>
       <c r="E7" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="F7" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G7" t="n">
-        <v>14.8</v>
+        <v>23.9</v>
       </c>
       <c r="H7" t="n">
         <v>72</v>
@@ -1106,7 +1106,7 @@
         <v>780</v>
       </c>
       <c r="J7" t="n">
-        <v>20.6</v>
+        <v>33.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-actualización SAT Río V - 2026-10-07 17:32 UTC
</commit_message>
<xml_diff>
--- a/sat_unificado_rio_v_triprovincial.xlsx
+++ b/sat_unificado_rio_v_triprovincial.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D2" t="n">
         <v>1.9</v>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.39</v>
+        <v>1.49</v>
       </c>
       <c r="D3" t="n">
         <v>2.4</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="D4" t="n">
         <v>2.5</v>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="D5" t="n">
         <v>2.8</v>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="D6" t="n">
         <v>2.8</v>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.15</v>
+        <v>1.19</v>
       </c>
       <c r="D8" t="n">
         <v>2.6</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="D9" t="n">
         <v>2.2</v>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -898,16 +898,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="F2" t="n">
-        <v>14.7</v>
+        <v>12.9</v>
       </c>
       <c r="G2" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="H2" t="n">
         <v>55</v>
@@ -916,7 +916,7 @@
         <v>680</v>
       </c>
       <c r="J2" t="n">
-        <v>45.5</v>
+        <v>41.1</v>
       </c>
     </row>
     <row r="3">
@@ -936,16 +936,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="F3" t="n">
-        <v>8.300000000000001</v>
+        <v>13.7</v>
       </c>
       <c r="G3" t="n">
-        <v>19.8</v>
+        <v>23.8</v>
       </c>
       <c r="H3" t="n">
         <v>68</v>
@@ -954,7 +954,7 @@
         <v>750</v>
       </c>
       <c r="J3" t="n">
-        <v>29.1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -974,16 +974,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16.9</v>
+        <v>15.5</v>
       </c>
       <c r="E4" t="n">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
       <c r="F4" t="n">
-        <v>3.6</v>
+        <v>16.3</v>
       </c>
       <c r="G4" t="n">
-        <v>22.8</v>
+        <v>33.4</v>
       </c>
       <c r="H4" t="n">
         <v>70</v>
@@ -992,7 +992,7 @@
         <v>770</v>
       </c>
       <c r="J4" t="n">
-        <v>32.6</v>
+        <v>47.7</v>
       </c>
     </row>
     <row r="5">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>16.8</v>
+        <v>10.4</v>
       </c>
       <c r="E5" t="n">
-        <v>8.699999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="F5" t="n">
-        <v>4.1</v>
+        <v>4.7</v>
       </c>
       <c r="G5" t="n">
-        <v>29.6</v>
+        <v>15.7</v>
       </c>
       <c r="H5" t="n">
         <v>75</v>
@@ -1030,7 +1030,7 @@
         <v>800</v>
       </c>
       <c r="J5" t="n">
-        <v>39.5</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="6">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16.5</v>
+        <v>10.2</v>
       </c>
       <c r="E6" t="n">
-        <v>13.9</v>
+        <v>2.5</v>
       </c>
       <c r="F6" t="n">
-        <v>4.9</v>
+        <v>8.5</v>
       </c>
       <c r="G6" t="n">
-        <v>35.3</v>
+        <v>21.2</v>
       </c>
       <c r="H6" t="n">
         <v>78</v>
@@ -1068,7 +1068,7 @@
         <v>820</v>
       </c>
       <c r="J6" t="n">
-        <v>45.3</v>
+        <v>27.2</v>
       </c>
     </row>
     <row r="7">
@@ -1088,16 +1088,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>17.3</v>
+        <v>13.7</v>
       </c>
       <c r="E7" t="n">
-        <v>2.1</v>
+        <v>1.1</v>
       </c>
       <c r="F7" t="n">
-        <v>4.5</v>
+        <v>8.6</v>
       </c>
       <c r="G7" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="H7" t="n">
         <v>72</v>
@@ -1106,7 +1106,7 @@
         <v>780</v>
       </c>
       <c r="J7" t="n">
-        <v>33.2</v>
+        <v>32.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>